<commit_message>
fix: remove average monthly values manual sections
</commit_message>
<xml_diff>
--- a/frontend/public/templates/rtm-ems-log-amv-template.xlsx
+++ b/frontend/public/templates/rtm-ems-log-amv-template.xlsx
@@ -454,23 +454,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Retrieval Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2">
-        <f>TODAY()</f>
-        <v/>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
           <t>Update Date</t>
         </is>
-      </c>
-      <c r="B2" s="2">
-        <f>TODAY()</f>
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -521,15 +506,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>10.25</v>
-      </c>
-      <c r="C5" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="H5" t="n">
-        <v>30.75</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -648,9 +624,6 @@
         <is>
           <t>1</t>
         </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1.25</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
fix: align AMV rollover with design
</commit_message>
<xml_diff>
--- a/frontend/public/templates/rtm-ems-log-amv-template.xlsx
+++ b/frontend/public/templates/rtm-ems-log-amv-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="R2ade46001d384e21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="R4de123c7489d4333"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -421,7 +421,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>Enter values for one month. Choose the effective month on the upload screen.</x:v>
+        <x:v>Enter values for the effective month shown on the upload screen.</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>

</xml_diff>

<commit_message>
fix: retire Grade A from RTM AMV
</commit_message>
<xml_diff>
--- a/frontend/public/templates/rtm-ems-log-amv-template.xlsx
+++ b/frontend/public/templates/rtm-ems-log-amv-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="R4de123c7489d4333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="R5275c03016df4281"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -421,7 +421,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>Enter values for the effective month shown on the upload screen.</x:v>
+        <x:v>Enter values for one month. Choose the effective month on the upload screen.</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>
@@ -459,7 +459,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="22" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="B3" s="28"/>
       <x:c r="C3" s="28"/>
@@ -471,7 +471,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="22" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="B4" s="28"/>
       <x:c r="C4" s="28"/>
@@ -483,7 +483,7 @@
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="22" t="str">
-        <x:v>C</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="B5" s="28"/>
       <x:c r="C5" s="28"/>
@@ -495,7 +495,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="22" t="str">
-        <x:v>D</x:v>
+        <x:v>E</x:v>
       </x:c>
       <x:c r="B6" s="28"/>
       <x:c r="C6" s="28"/>
@@ -507,7 +507,7 @@
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="22" t="str">
-        <x:v>E</x:v>
+        <x:v>F</x:v>
       </x:c>
       <x:c r="B7" s="28"/>
       <x:c r="C7" s="28"/>
@@ -519,7 +519,7 @@
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="22" t="str">
-        <x:v>F</x:v>
+        <x:v>G</x:v>
       </x:c>
       <x:c r="B8" s="28"/>
       <x:c r="C8" s="28"/>
@@ -531,7 +531,7 @@
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="22" t="str">
-        <x:v>G</x:v>
+        <x:v>H</x:v>
       </x:c>
       <x:c r="B9" s="28"/>
       <x:c r="C9" s="28"/>
@@ -543,7 +543,7 @@
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="22" t="str">
-        <x:v>H</x:v>
+        <x:v>I</x:v>
       </x:c>
       <x:c r="B10" s="28"/>
       <x:c r="C10" s="28"/>
@@ -555,7 +555,7 @@
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="22" t="str">
-        <x:v>I</x:v>
+        <x:v>J</x:v>
       </x:c>
       <x:c r="B11" s="28"/>
       <x:c r="C11" s="28"/>
@@ -567,7 +567,7 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="22" t="str">
-        <x:v>J</x:v>
+        <x:v>K</x:v>
       </x:c>
       <x:c r="B12" s="28"/>
       <x:c r="C12" s="28"/>
@@ -579,7 +579,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="22" t="str">
-        <x:v>K</x:v>
+        <x:v>L</x:v>
       </x:c>
       <x:c r="B13" s="28"/>
       <x:c r="C13" s="28"/>
@@ -591,7 +591,7 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="22" t="str">
-        <x:v>L</x:v>
+        <x:v>M</x:v>
       </x:c>
       <x:c r="B14" s="28"/>
       <x:c r="C14" s="28"/>
@@ -603,7 +603,7 @@
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="22" t="str">
-        <x:v>M</x:v>
+        <x:v>U</x:v>
       </x:c>
       <x:c r="B15" s="28"/>
       <x:c r="C15" s="28"/>
@@ -615,7 +615,7 @@
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="22" t="str">
-        <x:v>U</x:v>
+        <x:v>X</x:v>
       </x:c>
       <x:c r="B16" s="28"/>
       <x:c r="C16" s="28"/>
@@ -627,7 +627,7 @@
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="22" t="str">
-        <x:v>X</x:v>
+        <x:v>Y</x:v>
       </x:c>
       <x:c r="B17" s="28"/>
       <x:c r="C17" s="28"/>
@@ -637,18 +637,6 @@
       <x:c r="G17" s="28"/>
       <x:c r="H17" s="28"/>
     </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="22" t="str">
-        <x:v>Y</x:v>
-      </x:c>
-      <x:c r="B18" s="28"/>
-      <x:c r="C18" s="28"/>
-      <x:c r="D18" s="28"/>
-      <x:c r="E18" s="28"/>
-      <x:c r="F18" s="28"/>
-      <x:c r="G18" s="28"/>
-      <x:c r="H18" s="28"/>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
fix: address RTM AMV testing feedback
</commit_message>
<xml_diff>
--- a/frontend/public/templates/rtm-ems-log-amv-template.xlsx
+++ b/frontend/public/templates/rtm-ems-log-amv-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="R5275c03016df4281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average market values" sheetId="1" r:id="Rc430822f65c54023"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -421,7 +421,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="9" t="str">
-        <x:v>Enter values for one month. Choose the effective month on the upload screen.</x:v>
+        <x:v>Enter values for month.</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>

</xml_diff>